<commit_message>
Fixed SD card mount traces
Ran SD card traces on bottom instead of top to avoid sd mount prohibition area
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevI/MusselGapeTracker_RevI_PurchaseList.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevI/MusselGapeTracker_RevI_PurchaseList.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Documents/GitHub/MusselGapeTracker_hardware/KiCad_files/MusselGapeTracker_RevI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837CC0D3-9025-F64E-A65B-8629E3A028DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781FA6FF-897B-9B4A-A077-27D12518E3AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1680" yWindow="1020" windowWidth="27640" windowHeight="16680" xr2:uid="{E7DEF6FF-2B66-CB45-A28F-80AEC1E72622}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -575,7 +575,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -605,13 +605,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1050,7 +1047,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="7">
@@ -1071,7 +1068,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="7">
@@ -1092,7 +1089,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="7">
@@ -1113,7 +1110,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="7">
@@ -1134,7 +1131,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="7">
@@ -1155,7 +1152,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="7">
@@ -1176,7 +1173,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="7">
@@ -1197,7 +1194,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="7">
@@ -1218,7 +1215,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="7">
@@ -1239,7 +1236,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B18" s="7">
@@ -1260,7 +1257,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="3" t="s">
         <v>139</v>
       </c>
       <c r="B19" s="7">
@@ -1281,7 +1278,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="7">
@@ -1302,7 +1299,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="7">
@@ -1323,7 +1320,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B22" s="7">
@@ -1344,7 +1341,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="7">
@@ -1365,7 +1362,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="7">
@@ -1386,7 +1383,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="7">
@@ -1407,7 +1404,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B26" s="7">
@@ -1428,7 +1425,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="16" t="s">
+      <c r="A27" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B27" s="7">
@@ -1449,7 +1446,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B28" s="7">
@@ -1470,7 +1467,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B29" s="7">
@@ -1491,7 +1488,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B30" s="7">
@@ -1512,7 +1509,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="3" t="s">
         <v>25</v>
       </c>
       <c r="B31" s="7">
@@ -1533,7 +1530,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B32" s="7">
@@ -1554,7 +1551,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B33" s="7">
@@ -1575,7 +1572,7 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B34" s="7">
@@ -1596,7 +1593,7 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B35" s="7">
@@ -1617,7 +1614,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="16" t="s">
         <v>30</v>
       </c>
       <c r="B36" s="7">
@@ -1638,7 +1635,7 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="3" t="s">
         <v>31</v>
       </c>
       <c r="B37" s="7">
@@ -1749,7 +1746,7 @@
       <c r="B42" s="7">
         <v>1</v>
       </c>
-      <c r="C42" s="24" t="s">
+      <c r="C42" s="23" t="s">
         <v>73</v>
       </c>
       <c r="D42" s="6">
@@ -1902,10 +1899,10 @@
       <c r="B54" s="7">
         <v>1</v>
       </c>
-      <c r="D54" s="21">
+      <c r="D54" s="20">
         <v>32.450000000000003</v>
       </c>
-      <c r="E54" s="21">
+      <c r="E54" s="20">
         <f>D54/3</f>
         <v>10.816666666666668</v>
       </c>
@@ -1920,10 +1917,10 @@
       <c r="B55" s="7">
         <v>16</v>
       </c>
-      <c r="D55" s="19">
+      <c r="D55" s="18">
         <v>0.5</v>
       </c>
-      <c r="E55" s="21">
+      <c r="E55" s="20">
         <f>D55*B55</f>
         <v>8</v>
       </c>
@@ -1936,7 +1933,7 @@
       <c r="B57" s="7"/>
       <c r="C57" s="13"/>
       <c r="D57" s="6"/>
-      <c r="E57" s="19"/>
+      <c r="E57" s="18"/>
       <c r="F57" s="14"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -1958,7 +1955,7 @@
       <c r="F59" s="14"/>
     </row>
     <row r="60" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A60" s="18" t="s">
+      <c r="A60" s="17" t="s">
         <v>2</v>
       </c>
       <c r="B60" s="7"/>
@@ -1974,13 +1971,13 @@
       <c r="B62" s="7">
         <v>3</v>
       </c>
-      <c r="C62" s="20" t="s">
+      <c r="C62" s="19" t="s">
         <v>92</v>
       </c>
       <c r="D62" s="6">
         <v>25.89</v>
       </c>
-      <c r="E62" s="19">
+      <c r="E62" s="18">
         <f>D62*B62</f>
         <v>77.67</v>
       </c>
@@ -1989,7 +1986,7 @@
       </c>
     </row>
     <row r="64" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A64" s="18" t="s">
+      <c r="A64" s="17" t="s">
         <v>82</v>
       </c>
       <c r="B64" s="7"/>
@@ -2009,7 +2006,7 @@
       <c r="D66" s="6">
         <v>38.950000000000003</v>
       </c>
-      <c r="E66" s="19">
+      <c r="E66" s="18">
         <f>D66*0</f>
         <v>0</v>
       </c>
@@ -2032,12 +2029,12 @@
       <c r="B68" s="7"/>
       <c r="C68" s="13"/>
       <c r="D68" s="6"/>
-      <c r="E68" s="19"/>
+      <c r="E68" s="18"/>
       <c r="F68" s="14"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
-      <c r="D69" s="22"/>
+      <c r="D69" s="21"/>
     </row>
     <row r="70" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
@@ -2046,10 +2043,10 @@
       <c r="B70" s="7">
         <v>1</v>
       </c>
-      <c r="D70" s="22">
+      <c r="D70" s="21">
         <v>12.4</v>
       </c>
-      <c r="E70" s="23">
+      <c r="E70" s="22">
         <f>D70*B70</f>
         <v>12.4</v>
       </c>
@@ -2064,10 +2061,10 @@
       <c r="B71" s="7">
         <v>1</v>
       </c>
-      <c r="D71" s="22">
+      <c r="D71" s="21">
         <v>5</v>
       </c>
-      <c r="E71" s="23">
+      <c r="E71" s="22">
         <f>D71*B71</f>
         <v>5</v>
       </c>
@@ -2076,7 +2073,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A72" s="18"/>
+      <c r="A72" s="17"/>
       <c r="B72" s="7"/>
       <c r="C72" s="2"/>
       <c r="D72" s="6"/>
@@ -2087,7 +2084,7 @@
       <c r="B74" s="7"/>
       <c r="C74" s="13"/>
       <c r="D74" s="6"/>
-      <c r="E74" s="19"/>
+      <c r="E74" s="18"/>
       <c r="F74" s="14"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
@@ -2095,23 +2092,23 @@
       <c r="B79" s="7"/>
       <c r="C79" s="13"/>
       <c r="D79" s="6"/>
-      <c r="E79" s="19"/>
+      <c r="E79" s="18"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
-      <c r="D80" s="22"/>
+      <c r="D80" s="21"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="7"/>
-      <c r="D81" s="22"/>
-      <c r="E81" s="23"/>
+      <c r="D81" s="21"/>
+      <c r="E81" s="22"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="7"/>
-      <c r="D82" s="22"/>
-      <c r="E82" s="23"/>
+      <c r="D82" s="21"/>
+      <c r="E82" s="22"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>